<commit_message>
Update World Calendar with revised events for Son's character development and truth-seeking journey.
</commit_message>
<xml_diff>
--- a/world_calendar.xlsx
+++ b/world_calendar.xlsx
@@ -1844,14 +1844,7 @@
     </r>
   </si>
   <si>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <color theme="1"/>
-        <sz val="11.0"/>
-      </rPr>
-      <t>Son bắt đầu đặt những câu hỏi đầu tiên về Elena.</t>
-    </r>
+    <t>Son bắt đầu tự mình đi tìm sự thật</t>
   </si>
   <si>
     <r>
@@ -5118,7 +5111,7 @@
         <v>189</v>
       </c>
       <c r="G55" s="1"/>
-      <c r="H55" s="1" t="s">
+      <c r="H55" s="2" t="s">
         <v>190</v>
       </c>
     </row>

</xml_diff>